<commit_message>
weekly weather data cleaning
</commit_message>
<xml_diff>
--- a/data/raw-data/Weekly_CSS_and_Environmental_Data.xlsx
+++ b/data/raw-data/Weekly_CSS_and_Environmental_Data.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dawsondeal/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esthe\Documents\GitHub\EstherPalmer-MADA-project\data\raw-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35EF86F3-B4BC-044E-A805-60E45AE283E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44CE4D76-EACE-4890-AA29-9CF8EA95A48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4280" yWindow="1900" windowWidth="24840" windowHeight="16180" activeTab="1" xr2:uid="{447D4815-5EE5-A74F-BEA3-77C832950E0E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{447D4815-5EE5-A74F-BEA3-77C832950E0E}"/>
   </bookViews>
   <sheets>
     <sheet name="CSS" sheetId="1" r:id="rId1"/>
     <sheet name="Weather" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -156,15 +156,6 @@
     <t>10'2"</t>
   </si>
   <si>
-    <t>9ft 10in</t>
-  </si>
-  <si>
-    <t>12ft 3in</t>
-  </si>
-  <si>
-    <t>10ft 0in</t>
-  </si>
-  <si>
     <t>8'11"</t>
   </si>
   <si>
@@ -187,6 +178,15 @@
   </si>
   <si>
     <t>9'10"</t>
+  </si>
+  <si>
+    <t>9' 10"</t>
+  </si>
+  <si>
+    <t>12' 3"</t>
+  </si>
+  <si>
+    <t>10' 0"</t>
   </si>
 </sst>
 </file>
@@ -562,9 +562,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37C8718A-142B-A64D-A8CE-47F52054126A}">
   <dimension ref="A1:Z14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.4">
       <c r="B1">
         <v>232</v>
       </c>
@@ -641,7 +641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -722,7 +722,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -803,7 +803,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -884,7 +884,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -965,7 +965,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1046,7 +1046,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1127,7 +1127,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1289,7 +1289,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1370,7 +1370,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1722,9 +1722,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E7D257-938C-9B48-8F46-DEBD53398B44}">
   <dimension ref="A1:Z16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.4">
       <c r="B1" t="s">
         <v>13</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>309</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>316</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>323</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>330</v>
       </c>
@@ -2121,7 +2121,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A6">
         <v>337</v>
       </c>
@@ -2162,7 +2162,7 @@
         <v>11</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="O6">
         <v>79</v>
@@ -2201,7 +2201,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A7">
         <v>344</v>
       </c>
@@ -2242,7 +2242,7 @@
         <v>11</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="O7">
         <v>78.2</v>
@@ -2281,7 +2281,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A8">
         <v>358</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>12</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="O8">
         <v>88.3</v>
@@ -2361,7 +2361,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>393</v>
       </c>
@@ -2402,7 +2402,7 @@
         <v>14</v>
       </c>
       <c r="N9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="O9">
         <v>93.6</v>
@@ -2441,7 +2441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>400</v>
       </c>
@@ -2482,7 +2482,7 @@
         <v>13</v>
       </c>
       <c r="N10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="O10">
         <v>91</v>
@@ -2521,7 +2521,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>407</v>
       </c>
@@ -2562,7 +2562,7 @@
         <v>19</v>
       </c>
       <c r="N11" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="O11">
         <v>95.8</v>
@@ -2601,7 +2601,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>414</v>
       </c>
@@ -2642,7 +2642,7 @@
         <v>16</v>
       </c>
       <c r="N12" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="O12">
         <v>94.4</v>
@@ -2663,7 +2663,7 @@
         <v>85.2</v>
       </c>
       <c r="U12" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="V12">
         <v>28.56</v>
@@ -2681,7 +2681,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>421</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="O13">
         <v>93.2</v>
@@ -2761,7 +2761,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>428</v>
       </c>
@@ -2799,10 +2799,10 @@
         <v>6.6666666666666666E-2</v>
       </c>
       <c r="M14" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="N14" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="O14">
         <v>98.7</v>
@@ -2841,7 +2841,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A15">
         <v>435</v>
       </c>
@@ -2921,7 +2921,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.4">
       <c r="A16">
         <v>442</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>19</v>
       </c>
       <c r="N16" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="O16">
         <v>81.599999999999994</v>

</xml_diff>

<commit_message>
test data actually here now
</commit_message>
<xml_diff>
--- a/data/raw-data/Weekly_CSS_and_Environmental_Data.xlsx
+++ b/data/raw-data/Weekly_CSS_and_Environmental_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esthe\Documents\GitHub\EstherPalmer-MADA-project\data\raw-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44CE4D76-EACE-4890-AA29-9CF8EA95A48D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D5CDFC6-3B0A-410A-BCF1-D09FB4D98FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{447D4815-5EE5-A74F-BEA3-77C832950E0E}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{447D4815-5EE5-A74F-BEA3-77C832950E0E}"/>
   </bookViews>
   <sheets>
     <sheet name="CSS" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="58">
   <si>
     <t>Frequency</t>
   </si>
@@ -187,6 +187,30 @@
   </si>
   <si>
     <t>10' 0"</t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t>7'5"</t>
+  </si>
+  <si>
+    <t>7'3"</t>
+  </si>
+  <si>
+    <t>7'6"</t>
+  </si>
+  <si>
+    <t>9'7"</t>
+  </si>
+  <si>
+    <t>8'6"</t>
+  </si>
+  <si>
+    <t>8'4"</t>
+  </si>
+  <si>
+    <t>9'2"</t>
   </si>
 </sst>
 </file>
@@ -1721,30 +1745,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E7D257-938C-9B48-8F46-DEBD53398B44}">
-  <dimension ref="A1:Z16"/>
+  <dimension ref="A1:Y27"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.4"/>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>50</v>
+      </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I1" t="s">
         <v>20</v>
@@ -1753,398 +1780,359 @@
         <v>20</v>
       </c>
       <c r="K1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="N1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="S1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="T1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="U1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="V1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="W1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="X1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Y1" t="s">
-        <v>34</v>
-      </c>
-      <c r="Z1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.4">
       <c r="A2">
-        <v>309</v>
+        <v>232</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>78.8</v>
       </c>
       <c r="C2">
-        <v>95.4</v>
+        <v>56.6</v>
       </c>
       <c r="D2">
-        <v>68.7</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>7.13</v>
       </c>
       <c r="F2">
-        <v>6.97</v>
+        <v>0.3</v>
       </c>
       <c r="G2">
+        <v>5.2</v>
+      </c>
+      <c r="H2">
         <v>0.2</v>
       </c>
-      <c r="H2">
-        <v>14.7</v>
-      </c>
       <c r="I2">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="J2">
-        <v>0.5</v>
-      </c>
-      <c r="K2">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="L2">
-        <v>0.46666666666666662</v>
-      </c>
-      <c r="M2">
-        <v>15.5</v>
-      </c>
-      <c r="N2" t="s">
-        <v>35</v>
+        <v>14</v>
+      </c>
+      <c r="M2" t="s">
+        <v>51</v>
+      </c>
+      <c r="N2">
+        <v>53</v>
       </c>
       <c r="O2">
-        <v>77.099999999999994</v>
+        <v>29.3</v>
       </c>
       <c r="P2">
-        <v>46.3</v>
+        <v>44</v>
       </c>
       <c r="Q2">
-        <v>59.6</v>
+        <v>40.4</v>
       </c>
       <c r="R2">
-        <v>64.599999999999994</v>
+        <v>40.9</v>
       </c>
       <c r="S2">
-        <v>64.099999999999994</v>
+        <v>42.5</v>
       </c>
       <c r="T2">
-        <v>62.9</v>
+        <v>4.5</v>
       </c>
       <c r="U2">
+        <v>13.53</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>0.04</v>
+      </c>
+      <c r="X2">
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>239</v>
+      </c>
+      <c r="B3">
+        <v>106.2</v>
+      </c>
+      <c r="C3">
+        <v>75.7</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>7.15</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>3.1</v>
+      </c>
+      <c r="H3">
+        <v>0.1</v>
+      </c>
+      <c r="I3">
+        <v>0.1</v>
+      </c>
+      <c r="J3">
+        <v>0.1</v>
+      </c>
+      <c r="L3">
+        <v>19</v>
+      </c>
+      <c r="M3" t="s">
+        <v>40</v>
+      </c>
+      <c r="N3">
+        <v>30.2</v>
+      </c>
+      <c r="O3">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="P3">
+        <v>58</v>
+      </c>
+      <c r="Q3">
+        <v>33.9</v>
+      </c>
+      <c r="R3">
+        <v>34.799999999999997</v>
+      </c>
+      <c r="S3">
+        <v>39</v>
+      </c>
+      <c r="T3">
+        <v>3.6</v>
+      </c>
+      <c r="U3">
+        <v>3.71</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
+        <v>0.01</v>
+      </c>
+      <c r="X3">
+        <v>2.19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A4">
+        <v>246</v>
+      </c>
+      <c r="B4">
+        <v>119.7</v>
+      </c>
+      <c r="C4">
+        <v>99.4</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>7.28</v>
+      </c>
+      <c r="F4">
+        <v>0.25</v>
+      </c>
+      <c r="G4">
+        <v>5.7</v>
+      </c>
+      <c r="H4">
+        <v>0.2</v>
+      </c>
+      <c r="I4">
+        <v>0.2</v>
+      </c>
+      <c r="J4">
+        <v>0.2</v>
+      </c>
+      <c r="L4">
+        <v>18</v>
+      </c>
+      <c r="M4" t="s">
+        <v>51</v>
+      </c>
+      <c r="N4">
+        <v>57.6</v>
+      </c>
+      <c r="O4">
+        <v>32.700000000000003</v>
+      </c>
+      <c r="P4">
+        <v>58</v>
+      </c>
+      <c r="Q4">
+        <v>43.4</v>
+      </c>
+      <c r="R4">
+        <v>43.6</v>
+      </c>
+      <c r="S4">
+        <v>44</v>
+      </c>
+      <c r="T4">
+        <v>3.9</v>
+      </c>
+      <c r="U4">
+        <v>15.1</v>
+      </c>
+      <c r="V4">
+        <v>0</v>
+      </c>
+      <c r="W4">
+        <v>0.06</v>
+      </c>
+      <c r="X4">
+        <v>2.14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A5">
+        <v>253</v>
+      </c>
+      <c r="B5">
+        <v>163</v>
+      </c>
+      <c r="C5">
+        <v>115</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>7.12</v>
+      </c>
+      <c r="F5">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>15.7</v>
+      </c>
+      <c r="H5">
+        <v>0.2</v>
+      </c>
+      <c r="I5">
+        <v>0.2</v>
+      </c>
+      <c r="J5">
+        <v>0.2</v>
+      </c>
+      <c r="L5">
+        <v>19</v>
+      </c>
+      <c r="M5" t="s">
+        <v>52</v>
+      </c>
+      <c r="N5">
+        <v>77.900000000000006</v>
+      </c>
+      <c r="O5">
+        <v>50.3</v>
+      </c>
+      <c r="P5">
+        <v>65.900000000000006</v>
+      </c>
+      <c r="Q5">
+        <v>57.4</v>
+      </c>
+      <c r="R5">
+        <v>58</v>
+      </c>
+      <c r="S5">
+        <v>57</v>
+      </c>
+      <c r="T5">
         <v>2.6</v>
       </c>
-      <c r="V2">
-        <v>23.96</v>
-      </c>
-      <c r="W2">
-        <v>0</v>
-      </c>
-      <c r="X2">
-        <v>0.16</v>
-      </c>
-      <c r="Y2">
-        <v>2.11</v>
-      </c>
-      <c r="Z2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A3">
-        <v>316</v>
-      </c>
-      <c r="B3">
-        <v>4</v>
-      </c>
-      <c r="C3">
-        <v>34.9</v>
-      </c>
-      <c r="D3">
-        <v>22.1</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>6.88</v>
-      </c>
-      <c r="G3">
-        <v>0.1</v>
-      </c>
-      <c r="H3">
-        <v>14.3</v>
-      </c>
-      <c r="I3">
-        <v>1.2</v>
-      </c>
-      <c r="J3">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="K3">
-        <v>1.2</v>
-      </c>
-      <c r="L3">
-        <v>1.1666666666666667</v>
-      </c>
-      <c r="M3">
-        <v>18</v>
-      </c>
-      <c r="N3" t="s">
-        <v>36</v>
-      </c>
-      <c r="O3">
-        <v>65.599999999999994</v>
-      </c>
-      <c r="P3">
-        <v>42.5</v>
-      </c>
-      <c r="Q3">
-        <v>59</v>
-      </c>
-      <c r="R3">
-        <v>61.3</v>
-      </c>
-      <c r="S3">
-        <v>61.3</v>
-      </c>
-      <c r="T3">
-        <v>62.4</v>
-      </c>
-      <c r="U3">
-        <v>4.5</v>
-      </c>
-      <c r="V3">
-        <v>25.88</v>
-      </c>
-      <c r="W3">
-        <v>0</v>
-      </c>
-      <c r="X3">
-        <v>0.16</v>
-      </c>
-      <c r="Y3">
-        <v>11.22</v>
-      </c>
-      <c r="Z3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A4">
-        <v>323</v>
-      </c>
-      <c r="B4">
-        <v>3</v>
-      </c>
-      <c r="C4">
-        <v>84.7</v>
-      </c>
-      <c r="D4">
-        <v>60.1</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>6.94</v>
-      </c>
-      <c r="G4">
-        <v>0.15</v>
-      </c>
-      <c r="H4">
-        <v>16.2</v>
-      </c>
-      <c r="I4">
-        <v>0.5</v>
-      </c>
-      <c r="J4">
-        <v>0.5</v>
-      </c>
-      <c r="K4">
-        <v>0.5</v>
-      </c>
-      <c r="L4">
-        <v>0.5</v>
-      </c>
-      <c r="M4">
-        <v>12.5</v>
-      </c>
-      <c r="N4" t="s">
-        <v>37</v>
-      </c>
-      <c r="O4">
-        <v>71</v>
-      </c>
-      <c r="P4">
-        <v>50.2</v>
-      </c>
-      <c r="Q4">
-        <v>43.2</v>
-      </c>
-      <c r="R4">
-        <v>67.3</v>
-      </c>
-      <c r="S4">
-        <v>66.8</v>
-      </c>
-      <c r="T4">
-        <v>66</v>
-      </c>
-      <c r="U4">
-        <v>6.8</v>
-      </c>
-      <c r="V4">
-        <v>24.34</v>
-      </c>
-      <c r="W4">
-        <v>0</v>
-      </c>
-      <c r="X4">
-        <v>0.18</v>
-      </c>
-      <c r="Y4">
-        <v>3.38</v>
-      </c>
-      <c r="Z4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A5">
-        <v>330</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>94.4</v>
-      </c>
-      <c r="D5">
-        <v>67</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
+      <c r="U5">
+        <v>15.03</v>
+      </c>
+      <c r="V5">
+        <v>0</v>
+      </c>
+      <c r="W5">
+        <v>0.08</v>
+      </c>
+      <c r="X5">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A6">
+        <v>260</v>
+      </c>
+      <c r="B6">
+        <v>88.6</v>
+      </c>
+      <c r="C6">
+        <v>63.2</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
         <v>7.16</v>
       </c>
-      <c r="G5">
-        <v>0.01</v>
-      </c>
-      <c r="H5">
-        <v>17.600000000000001</v>
-      </c>
-      <c r="I5">
-        <v>0.4</v>
-      </c>
-      <c r="J5">
-        <v>0.4</v>
-      </c>
-      <c r="K5">
-        <v>0.4</v>
-      </c>
-      <c r="L5">
-        <v>0.40000000000000008</v>
-      </c>
-      <c r="M5">
-        <v>14.5</v>
-      </c>
-      <c r="N5" t="s">
-        <v>38</v>
-      </c>
-      <c r="O5">
-        <v>76</v>
-      </c>
-      <c r="P5">
-        <v>63.4</v>
-      </c>
-      <c r="Q5">
-        <v>78.400000000000006</v>
-      </c>
-      <c r="R5">
-        <v>72</v>
-      </c>
-      <c r="S5">
-        <v>71.7</v>
-      </c>
-      <c r="T5">
-        <v>71.400000000000006</v>
-      </c>
-      <c r="U5">
-        <v>2.5</v>
-      </c>
-      <c r="V5">
-        <v>12.31</v>
-      </c>
-      <c r="W5">
-        <v>0.03</v>
-      </c>
-      <c r="X5">
-        <v>0.1</v>
-      </c>
-      <c r="Y5">
-        <v>2.74</v>
-      </c>
-      <c r="Z5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A6">
-        <v>337</v>
-      </c>
-      <c r="B6">
-        <v>4</v>
-      </c>
-      <c r="C6">
-        <v>102.1</v>
-      </c>
-      <c r="D6">
-        <v>73</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
       <c r="F6">
-        <v>7.11</v>
+        <v>0.21</v>
       </c>
       <c r="G6">
-        <v>0.19</v>
+        <v>11.1</v>
       </c>
       <c r="H6">
-        <v>17.899999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="I6">
         <v>0.2</v>
@@ -2152,852 +2140,1621 @@
       <c r="J6">
         <v>0.2</v>
       </c>
-      <c r="K6">
+      <c r="L6">
+        <v>18.5</v>
+      </c>
+      <c r="M6" t="s">
+        <v>43</v>
+      </c>
+      <c r="N6">
+        <v>49</v>
+      </c>
+      <c r="O6">
+        <v>36.4</v>
+      </c>
+      <c r="P6">
+        <v>88.2</v>
+      </c>
+      <c r="Q6">
+        <v>51.1</v>
+      </c>
+      <c r="R6">
+        <v>52.1</v>
+      </c>
+      <c r="S6">
+        <v>55.6</v>
+      </c>
+      <c r="T6">
+        <v>4.2</v>
+      </c>
+      <c r="U6">
+        <v>1.6</v>
+      </c>
+      <c r="V6">
+        <v>0.16</v>
+      </c>
+      <c r="W6">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A7">
+        <v>267</v>
+      </c>
+      <c r="B7">
+        <v>124.5</v>
+      </c>
+      <c r="C7">
+        <v>87.3</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>6.95</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>7.3</v>
+      </c>
+      <c r="H7">
+        <v>0.4</v>
+      </c>
+      <c r="I7">
+        <v>0.4</v>
+      </c>
+      <c r="J7">
+        <v>0.5</v>
+      </c>
+      <c r="L7">
+        <v>19</v>
+      </c>
+      <c r="M7" t="s">
+        <v>53</v>
+      </c>
+      <c r="N7">
+        <v>57.9</v>
+      </c>
+      <c r="O7">
+        <v>26.8</v>
+      </c>
+      <c r="P7">
+        <v>56.5</v>
+      </c>
+      <c r="Q7">
+        <v>45.7</v>
+      </c>
+      <c r="R7">
+        <v>45.9</v>
+      </c>
+      <c r="S7">
+        <v>47</v>
+      </c>
+      <c r="T7" t="s">
+        <v>42</v>
+      </c>
+      <c r="U7">
+        <v>14.48</v>
+      </c>
+      <c r="V7">
+        <v>0</v>
+      </c>
+      <c r="W7">
+        <v>0.06</v>
+      </c>
+      <c r="X7">
+        <v>6.53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A8">
+        <v>274</v>
+      </c>
+      <c r="B8">
+        <v>115.2</v>
+      </c>
+      <c r="C8">
+        <v>82.3</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>6.93</v>
+      </c>
+      <c r="F8">
+        <v>0.18</v>
+      </c>
+      <c r="G8">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="H8">
         <v>0.2</v>
       </c>
-      <c r="L6">
-        <v>0.20000000000000004</v>
-      </c>
-      <c r="M6">
-        <v>11</v>
-      </c>
-      <c r="N6" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="O6">
-        <v>79</v>
-      </c>
-      <c r="P6">
-        <v>59.2</v>
-      </c>
-      <c r="Q6">
-        <v>72.099999999999994</v>
-      </c>
-      <c r="R6">
-        <v>74.099999999999994</v>
-      </c>
-      <c r="S6">
-        <v>73.099999999999994</v>
-      </c>
-      <c r="T6">
-        <v>71.599999999999994</v>
-      </c>
-      <c r="U6">
-        <v>2.5</v>
-      </c>
-      <c r="V6">
-        <v>26.54</v>
-      </c>
-      <c r="W6">
-        <v>0</v>
-      </c>
-      <c r="X6">
-        <v>0.21</v>
-      </c>
-      <c r="Y6">
-        <v>2.91</v>
-      </c>
-      <c r="Z6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A7">
-        <v>344</v>
-      </c>
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7">
-        <v>95.5</v>
-      </c>
-      <c r="D7">
-        <v>66</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>7.14</v>
-      </c>
-      <c r="G7">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="H7">
-        <v>15.3</v>
-      </c>
-      <c r="I7">
-        <v>0.3</v>
-      </c>
-      <c r="J7">
+      <c r="I8">
         <v>0.2</v>
-      </c>
-      <c r="K7">
-        <v>0.2</v>
-      </c>
-      <c r="L7">
-        <v>0.23333333333333331</v>
-      </c>
-      <c r="M7">
-        <v>11</v>
-      </c>
-      <c r="N7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="O7">
-        <v>78.2</v>
-      </c>
-      <c r="P7">
-        <v>47.3</v>
-      </c>
-      <c r="Q7">
-        <v>65.400000000000006</v>
-      </c>
-      <c r="R7">
-        <v>70.599999999999994</v>
-      </c>
-      <c r="S7">
-        <v>69.400000000000006</v>
-      </c>
-      <c r="T7">
-        <v>68.400000000000006</v>
-      </c>
-      <c r="U7">
-        <v>1.9</v>
-      </c>
-      <c r="V7">
-        <v>29.09</v>
-      </c>
-      <c r="W7">
-        <v>0</v>
-      </c>
-      <c r="X7">
-        <v>0.22</v>
-      </c>
-      <c r="Y7">
-        <v>5.92</v>
-      </c>
-      <c r="Z7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A8">
-        <v>358</v>
-      </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="C8">
-        <v>76.900000000000006</v>
-      </c>
-      <c r="D8">
-        <v>55.1</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>7.2</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>20.5</v>
-      </c>
-      <c r="I8">
-        <v>0.1</v>
       </c>
       <c r="J8">
         <v>0.2</v>
       </c>
-      <c r="K8">
+      <c r="L8">
+        <v>16.5</v>
+      </c>
+      <c r="M8" t="s">
+        <v>43</v>
+      </c>
+      <c r="N8">
+        <v>73.400000000000006</v>
+      </c>
+      <c r="O8">
+        <v>36.5</v>
+      </c>
+      <c r="P8">
+        <v>52.5</v>
+      </c>
+      <c r="Q8">
+        <v>53.4</v>
+      </c>
+      <c r="R8">
+        <v>53</v>
+      </c>
+      <c r="S8">
+        <v>51.2</v>
+      </c>
+      <c r="T8">
+        <v>2.9</v>
+      </c>
+      <c r="U8">
+        <v>19.3</v>
+      </c>
+      <c r="V8">
+        <v>0</v>
+      </c>
+      <c r="W8">
+        <v>0.11</v>
+      </c>
+      <c r="X8">
+        <v>2.77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A9">
+        <v>281</v>
+      </c>
+      <c r="B9">
+        <v>86.5</v>
+      </c>
+      <c r="C9">
+        <v>61.6</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>7.12</v>
+      </c>
+      <c r="F9">
+        <v>0.31</v>
+      </c>
+      <c r="G9">
+        <v>10.1</v>
+      </c>
+      <c r="H9">
+        <v>0.2</v>
+      </c>
+      <c r="I9">
+        <v>0.2</v>
+      </c>
+      <c r="J9">
+        <v>0.2</v>
+      </c>
+      <c r="L9">
+        <v>14</v>
+      </c>
+      <c r="M9" t="s">
+        <v>54</v>
+      </c>
+      <c r="N9">
+        <v>68</v>
+      </c>
+      <c r="O9">
+        <v>35.799999999999997</v>
+      </c>
+      <c r="P9">
+        <v>61.9</v>
+      </c>
+      <c r="Q9">
+        <v>52.7</v>
+      </c>
+      <c r="R9">
+        <v>52.4</v>
+      </c>
+      <c r="S9">
+        <v>52.5</v>
+      </c>
+      <c r="T9">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="U9">
+        <v>8.2799999999999994</v>
+      </c>
+      <c r="V9">
+        <v>0</v>
+      </c>
+      <c r="W9">
+        <v>0.05</v>
+      </c>
+      <c r="X9">
+        <v>2.2400000000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A10">
+        <v>288</v>
+      </c>
+      <c r="B10">
+        <v>70.900000000000006</v>
+      </c>
+      <c r="C10">
+        <v>50.4</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>6.96</v>
+      </c>
+      <c r="F10">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="G10">
+        <v>8.6</v>
+      </c>
+      <c r="H10">
+        <v>0.5</v>
+      </c>
+      <c r="I10">
+        <v>0.5</v>
+      </c>
+      <c r="J10">
+        <v>0.5</v>
+      </c>
+      <c r="L10">
+        <v>17.5</v>
+      </c>
+      <c r="M10" t="s">
+        <v>55</v>
+      </c>
+      <c r="N10">
+        <v>73.5</v>
+      </c>
+      <c r="O10">
+        <v>37.6</v>
+      </c>
+      <c r="P10">
+        <v>53.7</v>
+      </c>
+      <c r="Q10">
+        <v>52.9</v>
+      </c>
+      <c r="R10">
+        <v>52.5</v>
+      </c>
+      <c r="S10">
+        <v>51.2</v>
+      </c>
+      <c r="T10">
+        <v>2.5</v>
+      </c>
+      <c r="U10">
+        <v>22.05</v>
+      </c>
+      <c r="V10">
+        <v>0.01</v>
+      </c>
+      <c r="W10">
+        <v>0.13</v>
+      </c>
+      <c r="X10">
+        <v>5.1100000000000003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A11">
+        <v>295</v>
+      </c>
+      <c r="B11">
+        <v>119.5</v>
+      </c>
+      <c r="C11">
+        <v>84.7</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>6.97</v>
+      </c>
+      <c r="F11">
+        <v>0.22</v>
+      </c>
+      <c r="G11">
+        <v>10.3</v>
+      </c>
+      <c r="H11">
+        <v>0.5</v>
+      </c>
+      <c r="I11">
+        <v>0.5</v>
+      </c>
+      <c r="J11">
+        <v>0.4</v>
+      </c>
+      <c r="L11">
+        <v>16</v>
+      </c>
+      <c r="M11" t="s">
+        <v>56</v>
+      </c>
+      <c r="N11">
+        <v>75</v>
+      </c>
+      <c r="O11">
+        <v>36.200000000000003</v>
+      </c>
+      <c r="P11">
+        <v>36.6</v>
+      </c>
+      <c r="Q11">
+        <v>57.8</v>
+      </c>
+      <c r="R11">
+        <v>57.4</v>
+      </c>
+      <c r="S11">
+        <v>56.9</v>
+      </c>
+      <c r="T11">
+        <v>2.5</v>
+      </c>
+      <c r="U11">
+        <v>23.3</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="X11">
+        <v>2.2200000000000002</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A12">
+        <v>302</v>
+      </c>
+      <c r="B12">
+        <v>116.6</v>
+      </c>
+      <c r="C12">
+        <v>82.9</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>7.02</v>
+      </c>
+      <c r="F12">
+        <v>0.32</v>
+      </c>
+      <c r="G12">
+        <v>11.3</v>
+      </c>
+      <c r="H12">
+        <v>0.4</v>
+      </c>
+      <c r="I12">
+        <v>0.4</v>
+      </c>
+      <c r="J12">
+        <v>0.4</v>
+      </c>
+      <c r="L12">
+        <v>15</v>
+      </c>
+      <c r="M12" t="s">
+        <v>57</v>
+      </c>
+      <c r="N12">
+        <v>76.900000000000006</v>
+      </c>
+      <c r="O12">
+        <v>40.799999999999997</v>
+      </c>
+      <c r="P12">
+        <v>44.9</v>
+      </c>
+      <c r="Q12">
+        <v>58.8</v>
+      </c>
+      <c r="R12">
+        <v>58.4</v>
+      </c>
+      <c r="S12">
+        <v>57.8</v>
+      </c>
+      <c r="T12">
+        <v>4.3</v>
+      </c>
+      <c r="U12">
+        <v>23.53</v>
+      </c>
+      <c r="V12">
+        <v>0.01</v>
+      </c>
+      <c r="W12">
+        <v>0.16</v>
+      </c>
+      <c r="X12">
+        <v>5.04</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A13">
+        <v>309</v>
+      </c>
+      <c r="B13">
+        <v>95.4</v>
+      </c>
+      <c r="C13">
+        <v>68.7</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>6.97</v>
+      </c>
+      <c r="F13">
+        <v>0.2</v>
+      </c>
+      <c r="G13">
+        <v>14.7</v>
+      </c>
+      <c r="H13">
+        <v>0.5</v>
+      </c>
+      <c r="I13">
+        <v>0.5</v>
+      </c>
+      <c r="J13">
+        <v>0.4</v>
+      </c>
+      <c r="K13">
+        <v>0.46666666666666662</v>
+      </c>
+      <c r="L13">
+        <v>15.5</v>
+      </c>
+      <c r="M13" t="s">
+        <v>35</v>
+      </c>
+      <c r="N13">
+        <v>77.099999999999994</v>
+      </c>
+      <c r="O13">
+        <v>46.3</v>
+      </c>
+      <c r="P13">
+        <v>59.6</v>
+      </c>
+      <c r="Q13">
+        <v>64.599999999999994</v>
+      </c>
+      <c r="R13">
+        <v>64.099999999999994</v>
+      </c>
+      <c r="S13">
+        <v>62.9</v>
+      </c>
+      <c r="T13">
+        <v>2.6</v>
+      </c>
+      <c r="U13">
+        <v>23.96</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0.16</v>
+      </c>
+      <c r="X13">
+        <v>2.11</v>
+      </c>
+      <c r="Y13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A14">
+        <v>316</v>
+      </c>
+      <c r="B14">
+        <v>34.9</v>
+      </c>
+      <c r="C14">
+        <v>22.1</v>
+      </c>
+      <c r="D14">
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <v>6.88</v>
+      </c>
+      <c r="F14">
+        <v>0.1</v>
+      </c>
+      <c r="G14">
+        <v>14.3</v>
+      </c>
+      <c r="H14">
+        <v>1.2</v>
+      </c>
+      <c r="I14">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="J14">
+        <v>1.2</v>
+      </c>
+      <c r="K14">
+        <v>1.1666666666666667</v>
+      </c>
+      <c r="L14">
+        <v>18</v>
+      </c>
+      <c r="M14" t="s">
+        <v>36</v>
+      </c>
+      <c r="N14">
+        <v>65.599999999999994</v>
+      </c>
+      <c r="O14">
+        <v>42.5</v>
+      </c>
+      <c r="P14">
+        <v>59</v>
+      </c>
+      <c r="Q14">
+        <v>61.3</v>
+      </c>
+      <c r="R14">
+        <v>61.3</v>
+      </c>
+      <c r="S14">
+        <v>62.4</v>
+      </c>
+      <c r="T14">
+        <v>4.5</v>
+      </c>
+      <c r="U14">
+        <v>25.88</v>
+      </c>
+      <c r="V14">
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <v>0.16</v>
+      </c>
+      <c r="X14">
+        <v>11.22</v>
+      </c>
+      <c r="Y14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A15">
+        <v>323</v>
+      </c>
+      <c r="B15">
+        <v>84.7</v>
+      </c>
+      <c r="C15">
+        <v>60.1</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
+        <v>6.94</v>
+      </c>
+      <c r="F15">
+        <v>0.15</v>
+      </c>
+      <c r="G15">
+        <v>16.2</v>
+      </c>
+      <c r="H15">
+        <v>0.5</v>
+      </c>
+      <c r="I15">
+        <v>0.5</v>
+      </c>
+      <c r="J15">
+        <v>0.5</v>
+      </c>
+      <c r="K15">
+        <v>0.5</v>
+      </c>
+      <c r="L15">
+        <v>12.5</v>
+      </c>
+      <c r="M15" t="s">
+        <v>37</v>
+      </c>
+      <c r="N15">
+        <v>71</v>
+      </c>
+      <c r="O15">
+        <v>50.2</v>
+      </c>
+      <c r="P15">
+        <v>43.2</v>
+      </c>
+      <c r="Q15">
+        <v>67.3</v>
+      </c>
+      <c r="R15">
+        <v>66.8</v>
+      </c>
+      <c r="S15">
+        <v>66</v>
+      </c>
+      <c r="T15">
+        <v>6.8</v>
+      </c>
+      <c r="U15">
+        <v>24.34</v>
+      </c>
+      <c r="V15">
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <v>0.18</v>
+      </c>
+      <c r="X15">
+        <v>3.38</v>
+      </c>
+      <c r="Y15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A16">
+        <v>330</v>
+      </c>
+      <c r="B16">
+        <v>94.4</v>
+      </c>
+      <c r="C16">
+        <v>67</v>
+      </c>
+      <c r="D16">
+        <v>0</v>
+      </c>
+      <c r="E16">
+        <v>7.16</v>
+      </c>
+      <c r="F16">
+        <v>0.01</v>
+      </c>
+      <c r="G16">
+        <v>17.600000000000001</v>
+      </c>
+      <c r="H16">
+        <v>0.4</v>
+      </c>
+      <c r="I16">
+        <v>0.4</v>
+      </c>
+      <c r="J16">
+        <v>0.4</v>
+      </c>
+      <c r="K16">
+        <v>0.40000000000000008</v>
+      </c>
+      <c r="L16">
+        <v>14.5</v>
+      </c>
+      <c r="M16" t="s">
+        <v>38</v>
+      </c>
+      <c r="N16">
+        <v>76</v>
+      </c>
+      <c r="O16">
+        <v>63.4</v>
+      </c>
+      <c r="P16">
+        <v>78.400000000000006</v>
+      </c>
+      <c r="Q16">
+        <v>72</v>
+      </c>
+      <c r="R16">
+        <v>71.7</v>
+      </c>
+      <c r="S16">
+        <v>71.400000000000006</v>
+      </c>
+      <c r="T16">
+        <v>2.5</v>
+      </c>
+      <c r="U16">
+        <v>12.31</v>
+      </c>
+      <c r="V16">
+        <v>0.03</v>
+      </c>
+      <c r="W16">
+        <v>0.1</v>
+      </c>
+      <c r="X16">
+        <v>2.74</v>
+      </c>
+      <c r="Y16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A17">
+        <v>337</v>
+      </c>
+      <c r="B17">
+        <v>102.1</v>
+      </c>
+      <c r="C17">
+        <v>73</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>7.11</v>
+      </c>
+      <c r="F17">
+        <v>0.19</v>
+      </c>
+      <c r="G17">
+        <v>17.899999999999999</v>
+      </c>
+      <c r="H17">
+        <v>0.2</v>
+      </c>
+      <c r="I17">
+        <v>0.2</v>
+      </c>
+      <c r="J17">
+        <v>0.2</v>
+      </c>
+      <c r="K17">
+        <v>0.20000000000000004</v>
+      </c>
+      <c r="L17">
+        <v>11</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="N17">
+        <v>79</v>
+      </c>
+      <c r="O17">
+        <v>59.2</v>
+      </c>
+      <c r="P17">
+        <v>72.099999999999994</v>
+      </c>
+      <c r="Q17">
+        <v>74.099999999999994</v>
+      </c>
+      <c r="R17">
+        <v>73.099999999999994</v>
+      </c>
+      <c r="S17">
+        <v>71.599999999999994</v>
+      </c>
+      <c r="T17">
+        <v>2.5</v>
+      </c>
+      <c r="U17">
+        <v>26.54</v>
+      </c>
+      <c r="V17">
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <v>0.21</v>
+      </c>
+      <c r="X17">
+        <v>2.91</v>
+      </c>
+      <c r="Y17">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A18">
+        <v>344</v>
+      </c>
+      <c r="B18">
+        <v>95.5</v>
+      </c>
+      <c r="C18">
+        <v>66</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>7.14</v>
+      </c>
+      <c r="F18">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="G18">
+        <v>15.3</v>
+      </c>
+      <c r="H18">
         <v>0.3</v>
       </c>
-      <c r="L8">
+      <c r="I18">
+        <v>0.2</v>
+      </c>
+      <c r="J18">
+        <v>0.2</v>
+      </c>
+      <c r="K18">
+        <v>0.23333333333333331</v>
+      </c>
+      <c r="L18">
+        <v>11</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="N18">
+        <v>78.2</v>
+      </c>
+      <c r="O18">
+        <v>47.3</v>
+      </c>
+      <c r="P18">
+        <v>65.400000000000006</v>
+      </c>
+      <c r="Q18">
+        <v>70.599999999999994</v>
+      </c>
+      <c r="R18">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="S18">
+        <v>68.400000000000006</v>
+      </c>
+      <c r="T18">
+        <v>1.9</v>
+      </c>
+      <c r="U18">
+        <v>29.09</v>
+      </c>
+      <c r="V18">
+        <v>0</v>
+      </c>
+      <c r="W18">
+        <v>0.22</v>
+      </c>
+      <c r="X18">
+        <v>5.92</v>
+      </c>
+      <c r="Y18">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A19">
+        <v>358</v>
+      </c>
+      <c r="B19">
+        <v>76.900000000000006</v>
+      </c>
+      <c r="C19">
+        <v>55.1</v>
+      </c>
+      <c r="D19">
+        <v>0</v>
+      </c>
+      <c r="E19">
+        <v>7.2</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+      <c r="G19">
+        <v>20.5</v>
+      </c>
+      <c r="H19">
+        <v>0.1</v>
+      </c>
+      <c r="I19">
+        <v>0.2</v>
+      </c>
+      <c r="J19">
+        <v>0.3</v>
+      </c>
+      <c r="K19">
         <v>0.20000000000000004</v>
       </c>
-      <c r="M8">
+      <c r="L19">
         <v>12</v>
       </c>
-      <c r="N8" s="1" t="s">
+      <c r="M19" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="O8">
+      <c r="N19">
         <v>88.3</v>
       </c>
-      <c r="P8">
+      <c r="O19">
         <v>70.400000000000006</v>
       </c>
-      <c r="Q8">
+      <c r="P19">
         <v>68.599999999999994</v>
       </c>
-      <c r="R8">
+      <c r="Q19">
         <v>82.3</v>
       </c>
-      <c r="S8">
+      <c r="R19">
         <v>79.900000000000006</v>
       </c>
-      <c r="T8">
+      <c r="S19">
         <v>77.7</v>
       </c>
-      <c r="U8">
+      <c r="T19">
         <v>3.6</v>
       </c>
-      <c r="V8">
+      <c r="U19">
         <v>27.24</v>
       </c>
-      <c r="W8">
-        <v>0</v>
-      </c>
-      <c r="X8">
+      <c r="V19">
+        <v>0</v>
+      </c>
+      <c r="W19">
         <v>0.25</v>
       </c>
-      <c r="Y8">
+      <c r="X19">
         <v>3.28</v>
       </c>
-      <c r="Z8">
+      <c r="Y19">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A9">
+    <row r="20" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A20">
         <v>393</v>
       </c>
-      <c r="B9">
+      <c r="B20">
+        <v>82.4</v>
+      </c>
+      <c r="C20">
+        <v>59.3</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>7.07</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>22.2</v>
+      </c>
+      <c r="H20">
+        <v>0.1</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>3.3333333333333333E-2</v>
+      </c>
+      <c r="L20">
+        <v>14</v>
+      </c>
+      <c r="M20" t="s">
+        <v>39</v>
+      </c>
+      <c r="N20">
+        <v>93.6</v>
+      </c>
+      <c r="O20">
+        <v>72.5</v>
+      </c>
+      <c r="P20">
+        <v>72.7</v>
+      </c>
+      <c r="Q20">
+        <v>88.3</v>
+      </c>
+      <c r="R20">
+        <v>86.6</v>
+      </c>
+      <c r="S20">
+        <v>85</v>
+      </c>
+      <c r="T20">
+        <v>1.2</v>
+      </c>
+      <c r="U20">
+        <v>24.93</v>
+      </c>
+      <c r="V20">
+        <v>0</v>
+      </c>
+      <c r="W20">
+        <v>0.24</v>
+      </c>
+      <c r="X20">
+        <v>2.86</v>
+      </c>
+      <c r="Y20">
         <v>4</v>
       </c>
-      <c r="C9">
-        <v>82.4</v>
-      </c>
-      <c r="D9">
-        <v>59.3</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>7.07</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>22.2</v>
-      </c>
-      <c r="I9">
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A21">
+        <v>400</v>
+      </c>
+      <c r="B21">
+        <v>88.9</v>
+      </c>
+      <c r="C21">
+        <v>63.4</v>
+      </c>
+      <c r="D21">
+        <v>0</v>
+      </c>
+      <c r="E21">
+        <v>7.16</v>
+      </c>
+      <c r="F21">
+        <v>0.09</v>
+      </c>
+      <c r="G21">
+        <v>22.5</v>
+      </c>
+      <c r="H21">
         <v>0.1</v>
       </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
-      <c r="L9">
-        <v>3.3333333333333333E-2</v>
-      </c>
-      <c r="M9">
-        <v>14</v>
-      </c>
-      <c r="N9" t="s">
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0.1</v>
+      </c>
+      <c r="K21">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="L21">
+        <v>13</v>
+      </c>
+      <c r="M21" t="s">
         <v>39</v>
       </c>
-      <c r="O9">
-        <v>93.6</v>
-      </c>
-      <c r="P9">
+      <c r="N21">
+        <v>91</v>
+      </c>
+      <c r="O21">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="P21">
+        <v>72.400000000000006</v>
+      </c>
+      <c r="Q21">
+        <v>90.2</v>
+      </c>
+      <c r="R21">
+        <v>89</v>
+      </c>
+      <c r="S21">
+        <v>87.8</v>
+      </c>
+      <c r="T21">
+        <v>2.4</v>
+      </c>
+      <c r="U21">
+        <v>22.17</v>
+      </c>
+      <c r="V21">
+        <v>0</v>
+      </c>
+      <c r="W21">
+        <v>0.21</v>
+      </c>
+      <c r="X21">
+        <v>3.61</v>
+      </c>
+      <c r="Y21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A22">
+        <v>407</v>
+      </c>
+      <c r="B22">
+        <v>75.8</v>
+      </c>
+      <c r="C22">
+        <v>54.9</v>
+      </c>
+      <c r="D22">
+        <v>0</v>
+      </c>
+      <c r="E22">
+        <v>7.16</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+      <c r="G22">
+        <v>22.6</v>
+      </c>
+      <c r="H22">
+        <v>0.1</v>
+      </c>
+      <c r="I22">
+        <v>0.1</v>
+      </c>
+      <c r="J22">
+        <v>0.1</v>
+      </c>
+      <c r="K22">
+        <v>0.10000000000000002</v>
+      </c>
+      <c r="L22">
+        <v>19</v>
+      </c>
+      <c r="M22" t="s">
+        <v>40</v>
+      </c>
+      <c r="N22">
+        <v>95.8</v>
+      </c>
+      <c r="O22">
+        <v>71.2</v>
+      </c>
+      <c r="P22">
+        <v>60.3</v>
+      </c>
+      <c r="Q22">
+        <v>91.6</v>
+      </c>
+      <c r="R22">
+        <v>90.1</v>
+      </c>
+      <c r="S22">
+        <v>88.9</v>
+      </c>
+      <c r="T22">
+        <v>1.8</v>
+      </c>
+      <c r="U22">
+        <v>22.9</v>
+      </c>
+      <c r="V22">
+        <v>0</v>
+      </c>
+      <c r="W22">
+        <v>0.23</v>
+      </c>
+      <c r="X22">
+        <v>2.7</v>
+      </c>
+      <c r="Y22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A23">
+        <v>414</v>
+      </c>
+      <c r="B23">
+        <v>73.599999999999994</v>
+      </c>
+      <c r="C23">
+        <v>53.2</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>7.1</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>23.5</v>
+      </c>
+      <c r="H23">
+        <v>0.1</v>
+      </c>
+      <c r="I23">
+        <v>0.2</v>
+      </c>
+      <c r="J23">
+        <v>0.1</v>
+      </c>
+      <c r="K23">
+        <v>0.13333333333333333</v>
+      </c>
+      <c r="L23">
+        <v>16</v>
+      </c>
+      <c r="M23" t="s">
+        <v>41</v>
+      </c>
+      <c r="N23">
+        <v>94.4</v>
+      </c>
+      <c r="O23">
+        <v>72</v>
+      </c>
+      <c r="P23">
+        <v>64.900000000000006</v>
+      </c>
+      <c r="Q23">
+        <v>87.6</v>
+      </c>
+      <c r="R23">
+        <v>87.7</v>
+      </c>
+      <c r="S23">
+        <v>85.2</v>
+      </c>
+      <c r="T23" t="s">
+        <v>42</v>
+      </c>
+      <c r="U23">
+        <v>28.56</v>
+      </c>
+      <c r="V23">
+        <v>0</v>
+      </c>
+      <c r="W23">
+        <v>0.28000000000000003</v>
+      </c>
+      <c r="X23">
+        <v>3.92</v>
+      </c>
+      <c r="Y23">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A24">
+        <v>421</v>
+      </c>
+      <c r="B24">
+        <v>76.900000000000006</v>
+      </c>
+      <c r="C24">
+        <v>56.3</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>7.21</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+      <c r="G24">
+        <v>24.2</v>
+      </c>
+      <c r="H24">
+        <v>0.1</v>
+      </c>
+      <c r="I24">
+        <v>0.1</v>
+      </c>
+      <c r="J24">
+        <v>0.1</v>
+      </c>
+      <c r="K24">
+        <v>0.10000000000000002</v>
+      </c>
+      <c r="L24">
+        <v>17</v>
+      </c>
+      <c r="M24" t="s">
+        <v>43</v>
+      </c>
+      <c r="N24">
+        <v>93.2</v>
+      </c>
+      <c r="O24">
+        <v>76</v>
+      </c>
+      <c r="P24">
+        <v>79.099999999999994</v>
+      </c>
+      <c r="Q24">
+        <v>88.1</v>
+      </c>
+      <c r="R24">
+        <v>86.6</v>
+      </c>
+      <c r="S24">
+        <v>87.7</v>
+      </c>
+      <c r="T24">
+        <v>2.6</v>
+      </c>
+      <c r="U24">
+        <v>17.46</v>
+      </c>
+      <c r="V24">
+        <v>0.75</v>
+      </c>
+      <c r="W24">
+        <v>0.16</v>
+      </c>
+      <c r="X24">
+        <v>3.08</v>
+      </c>
+      <c r="Y24">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A25">
+        <v>428</v>
+      </c>
+      <c r="B25">
+        <v>87.1</v>
+      </c>
+      <c r="C25">
+        <v>63.9</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="E25">
+        <v>7.47</v>
+      </c>
+      <c r="F25">
+        <v>0.01</v>
+      </c>
+      <c r="G25">
+        <v>24.6</v>
+      </c>
+      <c r="H25">
+        <v>0.1</v>
+      </c>
+      <c r="I25">
+        <v>0.1</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="L25" t="s">
+        <v>44</v>
+      </c>
+      <c r="M25" t="s">
+        <v>45</v>
+      </c>
+      <c r="N25">
+        <v>98.7</v>
+      </c>
+      <c r="O25">
+        <v>76</v>
+      </c>
+      <c r="P25">
+        <v>71.3</v>
+      </c>
+      <c r="Q25">
+        <v>92.2</v>
+      </c>
+      <c r="R25">
+        <v>88.9</v>
+      </c>
+      <c r="S25">
+        <v>89.8</v>
+      </c>
+      <c r="T25">
+        <v>2</v>
+      </c>
+      <c r="U25">
+        <v>23.78</v>
+      </c>
+      <c r="V25">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="W25">
+        <v>0.23</v>
+      </c>
+      <c r="X25">
+        <v>12.49</v>
+      </c>
+      <c r="Y25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A26">
+        <v>435</v>
+      </c>
+      <c r="B26">
+        <v>57.6</v>
+      </c>
+      <c r="C26">
+        <v>53.7</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>7.05</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="H26">
+        <v>0.8</v>
+      </c>
+      <c r="I26">
+        <v>0.8</v>
+      </c>
+      <c r="J26">
+        <v>0.8</v>
+      </c>
+      <c r="K26">
+        <v>0.80000000000000016</v>
+      </c>
+      <c r="L26">
+        <v>18</v>
+      </c>
+      <c r="M26" t="s">
+        <v>36</v>
+      </c>
+      <c r="N26">
+        <v>65.900000000000006</v>
+      </c>
+      <c r="O26">
+        <v>63.8</v>
+      </c>
+      <c r="P26">
+        <v>97.6</v>
+      </c>
+      <c r="Q26">
+        <v>68.900000000000006</v>
+      </c>
+      <c r="R26">
+        <v>70.400000000000006</v>
+      </c>
+      <c r="S26">
+        <v>71.5</v>
+      </c>
+      <c r="T26">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="U26">
+        <v>3.52</v>
+      </c>
+      <c r="V26">
+        <v>0.83</v>
+      </c>
+      <c r="W26">
+        <v>0.03</v>
+      </c>
+      <c r="X26">
+        <v>12.41</v>
+      </c>
+      <c r="Y26">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.4">
+      <c r="A27">
+        <v>442</v>
+      </c>
+      <c r="B27">
+        <v>78.8</v>
+      </c>
+      <c r="C27">
+        <v>54.7</v>
+      </c>
+      <c r="D27">
+        <v>0</v>
+      </c>
+      <c r="E27">
+        <v>7</v>
+      </c>
+      <c r="F27">
+        <v>0.22</v>
+      </c>
+      <c r="G27">
+        <v>22.3</v>
+      </c>
+      <c r="H27">
+        <v>0.8</v>
+      </c>
+      <c r="I27">
+        <v>0.6</v>
+      </c>
+      <c r="J27">
+        <v>0.7</v>
+      </c>
+      <c r="K27">
+        <v>0.69999999999999984</v>
+      </c>
+      <c r="L27">
+        <v>19</v>
+      </c>
+      <c r="M27" t="s">
+        <v>46</v>
+      </c>
+      <c r="N27">
+        <v>81.599999999999994</v>
+      </c>
+      <c r="O27">
         <v>72.5</v>
       </c>
-      <c r="Q9">
-        <v>72.7</v>
-      </c>
-      <c r="R9">
-        <v>88.3</v>
-      </c>
-      <c r="S9">
-        <v>86.6</v>
-      </c>
-      <c r="T9">
-        <v>85</v>
-      </c>
-      <c r="U9">
-        <v>1.2</v>
-      </c>
-      <c r="V9">
-        <v>24.93</v>
-      </c>
-      <c r="W9">
-        <v>0</v>
-      </c>
-      <c r="X9">
-        <v>0.24</v>
-      </c>
-      <c r="Y9">
-        <v>2.86</v>
-      </c>
-      <c r="Z9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A10">
-        <v>400</v>
-      </c>
-      <c r="B10">
-        <v>3</v>
-      </c>
-      <c r="C10">
-        <v>88.9</v>
-      </c>
-      <c r="D10">
-        <v>63.4</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>7.16</v>
-      </c>
-      <c r="G10">
-        <v>0.09</v>
-      </c>
-      <c r="H10">
-        <v>22.5</v>
-      </c>
-      <c r="I10">
-        <v>0.1</v>
-      </c>
-      <c r="J10">
-        <v>0</v>
-      </c>
-      <c r="K10">
-        <v>0.1</v>
-      </c>
-      <c r="L10">
-        <v>6.6666666666666666E-2</v>
-      </c>
-      <c r="M10">
-        <v>13</v>
-      </c>
-      <c r="N10" t="s">
-        <v>39</v>
-      </c>
-      <c r="O10">
-        <v>91</v>
-      </c>
-      <c r="P10">
-        <v>71.099999999999994</v>
-      </c>
-      <c r="Q10">
-        <v>72.400000000000006</v>
-      </c>
-      <c r="R10">
-        <v>90.2</v>
-      </c>
-      <c r="S10">
-        <v>89</v>
-      </c>
-      <c r="T10">
-        <v>87.8</v>
-      </c>
-      <c r="U10">
-        <v>2.4</v>
-      </c>
-      <c r="V10">
-        <v>22.17</v>
-      </c>
-      <c r="W10">
-        <v>0</v>
-      </c>
-      <c r="X10">
-        <v>0.21</v>
-      </c>
-      <c r="Y10">
-        <v>3.61</v>
-      </c>
-      <c r="Z10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A11">
-        <v>407</v>
-      </c>
-      <c r="B11">
-        <v>3</v>
-      </c>
-      <c r="C11">
-        <v>75.8</v>
-      </c>
-      <c r="D11">
-        <v>54.9</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>7.16</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>22.6</v>
-      </c>
-      <c r="I11">
-        <v>0.1</v>
-      </c>
-      <c r="J11">
-        <v>0.1</v>
-      </c>
-      <c r="K11">
-        <v>0.1</v>
-      </c>
-      <c r="L11">
-        <v>0.10000000000000002</v>
-      </c>
-      <c r="M11">
-        <v>19</v>
-      </c>
-      <c r="N11" t="s">
-        <v>40</v>
-      </c>
-      <c r="O11">
-        <v>95.8</v>
-      </c>
-      <c r="P11">
-        <v>71.2</v>
-      </c>
-      <c r="Q11">
-        <v>60.3</v>
-      </c>
-      <c r="R11">
-        <v>91.6</v>
-      </c>
-      <c r="S11">
-        <v>90.1</v>
-      </c>
-      <c r="T11">
-        <v>88.9</v>
-      </c>
-      <c r="U11">
-        <v>1.8</v>
-      </c>
-      <c r="V11">
-        <v>22.9</v>
-      </c>
-      <c r="W11">
-        <v>0</v>
-      </c>
-      <c r="X11">
-        <v>0.23</v>
-      </c>
-      <c r="Y11">
-        <v>2.7</v>
-      </c>
-      <c r="Z11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A12">
-        <v>414</v>
-      </c>
-      <c r="B12">
-        <v>5</v>
-      </c>
-      <c r="C12">
-        <v>73.599999999999994</v>
-      </c>
-      <c r="D12">
-        <v>53.2</v>
-      </c>
-      <c r="E12">
-        <v>0</v>
-      </c>
-      <c r="F12">
-        <v>7.1</v>
-      </c>
-      <c r="G12">
-        <v>0</v>
-      </c>
-      <c r="H12">
-        <v>23.5</v>
-      </c>
-      <c r="I12">
-        <v>0.1</v>
-      </c>
-      <c r="J12">
-        <v>0.2</v>
-      </c>
-      <c r="K12">
-        <v>0.1</v>
-      </c>
-      <c r="L12">
-        <v>0.13333333333333333</v>
-      </c>
-      <c r="M12">
-        <v>16</v>
-      </c>
-      <c r="N12" t="s">
-        <v>41</v>
-      </c>
-      <c r="O12">
-        <v>94.4</v>
-      </c>
-      <c r="P12">
-        <v>72</v>
-      </c>
-      <c r="Q12">
-        <v>64.900000000000006</v>
-      </c>
-      <c r="R12">
-        <v>87.6</v>
-      </c>
-      <c r="S12">
-        <v>87.7</v>
-      </c>
-      <c r="T12">
-        <v>85.2</v>
-      </c>
-      <c r="U12" t="s">
-        <v>42</v>
-      </c>
-      <c r="V12">
-        <v>28.56</v>
-      </c>
-      <c r="W12">
-        <v>0</v>
-      </c>
-      <c r="X12">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="Y12">
-        <v>3.92</v>
-      </c>
-      <c r="Z12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A13">
-        <v>421</v>
-      </c>
-      <c r="B13">
-        <v>4</v>
-      </c>
-      <c r="C13">
-        <v>76.900000000000006</v>
-      </c>
-      <c r="D13">
-        <v>56.3</v>
-      </c>
-      <c r="E13">
-        <v>0</v>
-      </c>
-      <c r="F13">
-        <v>7.21</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>24.2</v>
-      </c>
-      <c r="I13">
-        <v>0.1</v>
-      </c>
-      <c r="J13">
-        <v>0.1</v>
-      </c>
-      <c r="K13">
-        <v>0.1</v>
-      </c>
-      <c r="L13">
-        <v>0.10000000000000002</v>
-      </c>
-      <c r="M13">
-        <v>17</v>
-      </c>
-      <c r="N13" t="s">
-        <v>43</v>
-      </c>
-      <c r="O13">
-        <v>93.2</v>
-      </c>
-      <c r="P13">
-        <v>76</v>
-      </c>
-      <c r="Q13">
-        <v>79.099999999999994</v>
-      </c>
-      <c r="R13">
-        <v>88.1</v>
-      </c>
-      <c r="S13">
-        <v>86.6</v>
-      </c>
-      <c r="T13">
-        <v>87.7</v>
-      </c>
-      <c r="U13">
-        <v>2.6</v>
-      </c>
-      <c r="V13">
-        <v>17.46</v>
-      </c>
-      <c r="W13">
-        <v>0.75</v>
-      </c>
-      <c r="X13">
-        <v>0.16</v>
-      </c>
-      <c r="Y13">
-        <v>3.08</v>
-      </c>
-      <c r="Z13">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A14">
-        <v>428</v>
-      </c>
-      <c r="B14">
-        <v>5</v>
-      </c>
-      <c r="C14">
-        <v>87.1</v>
-      </c>
-      <c r="D14">
-        <v>63.9</v>
-      </c>
-      <c r="E14">
-        <v>0</v>
-      </c>
-      <c r="F14">
-        <v>7.47</v>
-      </c>
-      <c r="G14">
-        <v>0.01</v>
-      </c>
-      <c r="H14">
-        <v>24.6</v>
-      </c>
-      <c r="I14">
-        <v>0.1</v>
-      </c>
-      <c r="J14">
-        <v>0.1</v>
-      </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14">
-        <v>6.6666666666666666E-2</v>
-      </c>
-      <c r="M14" t="s">
-        <v>44</v>
-      </c>
-      <c r="N14" t="s">
-        <v>45</v>
-      </c>
-      <c r="O14">
-        <v>98.7</v>
-      </c>
-      <c r="P14">
-        <v>76</v>
-      </c>
-      <c r="Q14">
-        <v>71.3</v>
-      </c>
-      <c r="R14">
-        <v>92.2</v>
-      </c>
-      <c r="S14">
-        <v>88.9</v>
-      </c>
-      <c r="T14">
-        <v>89.8</v>
-      </c>
-      <c r="U14">
-        <v>2</v>
-      </c>
-      <c r="V14">
-        <v>23.78</v>
-      </c>
-      <c r="W14">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="X14">
-        <v>0.23</v>
-      </c>
-      <c r="Y14">
-        <v>12.49</v>
-      </c>
-      <c r="Z14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A15">
-        <v>435</v>
-      </c>
-      <c r="B15">
-        <v>4</v>
-      </c>
-      <c r="C15">
-        <v>57.6</v>
-      </c>
-      <c r="D15">
-        <v>53.7</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>7.05</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="H15">
-        <v>20.100000000000001</v>
-      </c>
-      <c r="I15">
-        <v>0.8</v>
-      </c>
-      <c r="J15">
-        <v>0.8</v>
-      </c>
-      <c r="K15">
-        <v>0.8</v>
-      </c>
-      <c r="L15">
-        <v>0.80000000000000016</v>
-      </c>
-      <c r="M15">
-        <v>18</v>
-      </c>
-      <c r="N15" t="s">
-        <v>36</v>
-      </c>
-      <c r="O15">
-        <v>65.900000000000006</v>
-      </c>
-      <c r="P15">
-        <v>63.8</v>
-      </c>
-      <c r="Q15">
-        <v>97.6</v>
-      </c>
-      <c r="R15">
-        <v>68.900000000000006</v>
-      </c>
-      <c r="S15">
-        <v>70.400000000000006</v>
-      </c>
-      <c r="T15">
-        <v>71.5</v>
-      </c>
-      <c r="U15">
-        <v>4.9000000000000004</v>
-      </c>
-      <c r="V15">
-        <v>3.52</v>
-      </c>
-      <c r="W15">
-        <v>0.83</v>
-      </c>
-      <c r="X15">
-        <v>0.03</v>
-      </c>
-      <c r="Y15">
-        <v>12.41</v>
-      </c>
-      <c r="Z15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A16">
-        <v>442</v>
-      </c>
-      <c r="B16">
-        <v>4</v>
-      </c>
-      <c r="C16">
-        <v>78.8</v>
-      </c>
-      <c r="D16">
-        <v>54.7</v>
-      </c>
-      <c r="E16">
-        <v>0</v>
-      </c>
-      <c r="F16">
-        <v>7</v>
-      </c>
-      <c r="G16">
-        <v>0.22</v>
-      </c>
-      <c r="H16">
-        <v>22.3</v>
-      </c>
-      <c r="I16">
-        <v>0.8</v>
-      </c>
-      <c r="J16">
-        <v>0.6</v>
-      </c>
-      <c r="K16">
-        <v>0.7</v>
-      </c>
-      <c r="L16">
-        <v>0.69999999999999984</v>
-      </c>
-      <c r="M16">
-        <v>19</v>
-      </c>
-      <c r="N16" t="s">
-        <v>46</v>
-      </c>
-      <c r="O16">
-        <v>81.599999999999994</v>
-      </c>
-      <c r="P16">
-        <v>72.5</v>
-      </c>
-      <c r="Q16">
+      <c r="P27">
         <v>92.8</v>
       </c>
-      <c r="R16">
+      <c r="Q27">
         <v>79</v>
       </c>
-      <c r="S16">
+      <c r="R27">
         <v>78.7</v>
       </c>
-      <c r="T16">
+      <c r="S27">
         <v>78</v>
       </c>
-      <c r="U16">
+      <c r="T27">
         <v>2.2000000000000002</v>
       </c>
-      <c r="V16">
+      <c r="U27">
         <v>12.89</v>
       </c>
-      <c r="W16">
+      <c r="V27">
         <v>0.44</v>
       </c>
-      <c r="X16">
+      <c r="W27">
         <v>0.11</v>
       </c>
-      <c r="Y16">
+      <c r="X27">
         <v>6.45</v>
       </c>
-      <c r="Z16">
+      <c r="Y27">
         <v>4</v>
       </c>
     </row>

</xml_diff>